<commit_message>
inclusão de sumários, finalização aula 5, modificação README
</commit_message>
<xml_diff>
--- a/Analise_de_dados_e_IA_Nivelamento/Semana_02/Funcoes_com_excel_operacoes_matematicas_e_filtros/05_Utilizando_outras_funcoes/db/Meteora Ecommerce - FINAL AULA 4.xlsx
+++ b/Analise_de_dados_e_IA_Nivelamento/Semana_02/Funcoes_com_excel_operacoes_matematicas_e_filtros/05_Utilizando_outras_funcoes/db/Meteora Ecommerce - FINAL AULA 4.xlsx
@@ -8,28 +8,29 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tlchaves\Documents\Santander\Santander-Imersao-Digital\Analise_de_dados_e_IA_Nivelamento\Semana_02\Funcoes_com_excel_operacoes_matematicas_e_filtros\05_Utilizando_outras_funcoes\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873631BE-9855-4AF2-9F6A-7D8C87F374B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE54BC1-68B6-4205-BBE2-3B9CD6A6600D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="5" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
   </bookViews>
   <sheets>
     <sheet name="Meu Gráfico" sheetId="6" state="hidden" r:id="rId1"/>
     <sheet name="Planilha3" sheetId="5" state="hidden" r:id="rId2"/>
-    <sheet name="Produtos" sheetId="1" r:id="rId3"/>
-    <sheet name="Planilha2" sheetId="11" r:id="rId4"/>
-    <sheet name="Produtos (Com Tabela)" sheetId="7" state="hidden" r:id="rId5"/>
-    <sheet name="Filtro Avançado" sheetId="9" state="hidden" r:id="rId6"/>
+    <sheet name="Produtos" sheetId="1" state="hidden" r:id="rId3"/>
+    <sheet name="Meus Números" sheetId="11" r:id="rId4"/>
+    <sheet name="Produtos (Com Tabela)" sheetId="7" r:id="rId5"/>
+    <sheet name="Meus Números (Tabela)" sheetId="12" r:id="rId6"/>
+    <sheet name="Filtro Avançado" sheetId="9" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Produtos!$A$3:$G$42</definedName>
-    <definedName name="_xlnm.Extract" localSheetId="5">'Filtro Avançado'!$B$6:$H$6</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="5">'Filtro Avançado'!$B$2:$C$3</definedName>
+    <definedName name="_xlnm.Extract" localSheetId="6">'Filtro Avançado'!$B$6:$H$6</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="6">'Filtro Avançado'!$B$2:$C$3</definedName>
     <definedName name="Int_Nome_Produtos">Produtos!$A$4:$A$42</definedName>
     <definedName name="Int_Quantidade">Produtos!$F$4:$F$42</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId7"/>
+    <pivotCache cacheId="0" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="43">
   <si>
     <t>Produtos</t>
   </si>
@@ -564,10 +565,14 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -583,7 +588,7 @@
       <alignment horizontal="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -675,6 +680,15 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -687,18 +701,25 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="19" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="10" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="11" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="14" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="19" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Cabeçalho Meteora" xfId="3" xr:uid="{43DBFFA1-791E-423B-B2A6-377CC2810274}"/>
@@ -2894,7 +2915,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3E8EAC5A-BA80-4829-83D6-590270917CF9}" name="Tabela1" displayName="Tabela1" ref="A3:G43" totalsRowCount="1" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3E8EAC5A-BA80-4829-83D6-590270917CF9}" name="TB_Produtos" displayName="TB_Produtos" ref="A3:G43" totalsRowCount="1" headerRowDxfId="16" dataDxfId="15" totalsRowDxfId="14">
   <autoFilter ref="A3:G42" xr:uid="{3E8EAC5A-BA80-4829-83D6-590270917CF9}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:G42">
     <sortCondition descending="1" ref="E3:E42"/>
@@ -2905,11 +2926,11 @@
     <tableColumn id="3" xr3:uid="{A22CAE73-04B1-4CDC-8BD6-598A47E705D3}" name="Categoria" totalsRowFunction="count" dataDxfId="9" totalsRowDxfId="8"/>
     <tableColumn id="4" xr3:uid="{4117345F-4534-47DC-9C4F-74226F1EEFE0}" name="Preço Unitário" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="6"/>
     <tableColumn id="5" xr3:uid="{6D0F01FA-272F-4735-BE66-47CEF233DD1F}" name="Preço c/ Desconto" totalsRowFunction="sum" dataDxfId="5" totalsRowDxfId="4">
-      <calculatedColumnFormula>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</calculatedColumnFormula>
+      <calculatedColumnFormula>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{8AE83115-B06D-4CB9-9EBB-681EFAE7DC61}" name="Qtd" totalsRowFunction="sum" dataDxfId="3" totalsRowDxfId="2"/>
     <tableColumn id="7" xr3:uid="{10AC4673-D907-4090-890F-B0DF4BA1F58B}" name="Valor Total" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
-      <calculatedColumnFormula>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</calculatedColumnFormula>
+      <calculatedColumnFormula>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3393,15 +3414,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
     </row>
     <row r="2" spans="1:9" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
@@ -4445,11 +4466,11 @@
       <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="41" t="s">
+      <c r="A44" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="43"/>
+      <c r="B44" s="45"/>
+      <c r="C44" s="46"/>
       <c r="D44" s="22">
         <f>SUM(D4:D42)</f>
         <v>5962.2999999999984</v>
@@ -4486,34 +4507,42 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="4" width="22" customWidth="1"/>
-    <col min="6" max="8" width="22" customWidth="1"/>
+    <col min="6" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="21.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="35" customFormat="1" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="53" t="s">
         <v>38</v>
       </c>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
     </row>
     <row r="2" spans="1:8" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="49" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="F2" s="45" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="47"/>
-      <c r="H2" s="46"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
+      <c r="F2" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="42"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="37" t="s">
+      <c r="B3" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="48" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="48" t="s">
         <v>42</v>
       </c>
       <c r="F3" s="37" t="s">
@@ -4535,24 +4564,28 @@
         <f>SUM(Produtos!F4:F42)</f>
         <v>183</v>
       </c>
-      <c r="D4" s="36"/>
+      <c r="D4" s="52">
+        <f>AVERAGE(Int_Quantidade)</f>
+        <v>4.6923076923076925</v>
+      </c>
       <c r="F4" s="36">
         <f>COUNTIF(Int_Nome_Produtos,F2)</f>
         <v>3</v>
       </c>
       <c r="G4" s="36">
         <f>SUMIF(Int_Nome_Produtos,F2,Int_Quantidade)</f>
-        <v>10</v>
-      </c>
-      <c r="H4" s="36">
-        <f>SUMIF(Int_Nome_Produtos,G2,Int_Quantidade)</f>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="H4" s="52">
+        <f>AVERAGEIF(Int_Nome_Produtos,F2,Int_Quantidade)</f>
+        <v>1.3333333333333333</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" showErrorMessage="1" errorTitle="Erro de Digitação" error="Este produto não está listado na tabela original." promptTitle="Mensagem de Entrada" prompt="Teste de mensagem de entrada._x000a_" sqref="F2" xr:uid="{2CB6E629-3F0C-4869-93A6-28DEC2C4EA8C}">
@@ -4579,15 +4612,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
     </row>
     <row r="2" spans="1:9" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
@@ -4638,14 +4671,14 @@
         <v>399.9</v>
       </c>
       <c r="E4" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>359.90999999999997</v>
       </c>
       <c r="F4" s="30">
         <v>3</v>
       </c>
       <c r="G4" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>1079.73</v>
       </c>
       <c r="I4" s="26">
@@ -4666,14 +4699,14 @@
         <v>349.9</v>
       </c>
       <c r="E5" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>314.90999999999997</v>
       </c>
       <c r="F5" s="30">
         <v>2</v>
       </c>
       <c r="G5" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>629.81999999999994</v>
       </c>
       <c r="I5" s="28"/>
@@ -4692,14 +4725,14 @@
         <v>302.89999999999998</v>
       </c>
       <c r="E6" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>272.60999999999996</v>
       </c>
       <c r="F6" s="30">
         <v>2</v>
       </c>
       <c r="G6" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>545.21999999999991</v>
       </c>
       <c r="I6" s="28"/>
@@ -4718,14 +4751,14 @@
         <v>300</v>
       </c>
       <c r="E7" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>270</v>
       </c>
       <c r="F7" s="30">
         <v>1</v>
       </c>
       <c r="G7" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>270</v>
       </c>
       <c r="I7" s="28"/>
@@ -4744,14 +4777,14 @@
         <v>299.89999999999998</v>
       </c>
       <c r="E8" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>269.90999999999997</v>
       </c>
       <c r="F8" s="30">
         <v>1</v>
       </c>
       <c r="G8" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>269.90999999999997</v>
       </c>
       <c r="I8" s="28"/>
@@ -4770,14 +4803,14 @@
         <v>299.89999999999998</v>
       </c>
       <c r="E9" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>269.90999999999997</v>
       </c>
       <c r="F9" s="30">
         <v>1</v>
       </c>
       <c r="G9" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>269.90999999999997</v>
       </c>
       <c r="I9" s="28"/>
@@ -4796,14 +4829,14 @@
         <v>259.89999999999998</v>
       </c>
       <c r="E10" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>233.90999999999997</v>
       </c>
       <c r="F10" s="30">
         <v>2</v>
       </c>
       <c r="G10" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>467.81999999999994</v>
       </c>
       <c r="I10" s="28"/>
@@ -4822,14 +4855,14 @@
         <v>259.89999999999998</v>
       </c>
       <c r="E11" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>233.90999999999997</v>
       </c>
       <c r="F11" s="30">
         <v>0</v>
       </c>
       <c r="G11" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>0</v>
       </c>
       <c r="I11" s="28"/>
@@ -4848,14 +4881,14 @@
         <v>259.89999999999998</v>
       </c>
       <c r="E12" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>233.90999999999997</v>
       </c>
       <c r="F12" s="30">
         <v>1</v>
       </c>
       <c r="G12" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>233.90999999999997</v>
       </c>
       <c r="I12" s="28"/>
@@ -4874,14 +4907,14 @@
         <v>259.89999999999998</v>
       </c>
       <c r="E13" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>233.90999999999997</v>
       </c>
       <c r="F13" s="30">
         <v>1</v>
       </c>
       <c r="G13" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>233.90999999999997</v>
       </c>
       <c r="I13" s="28"/>
@@ -4900,14 +4933,14 @@
         <v>255</v>
       </c>
       <c r="E14" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>229.5</v>
       </c>
       <c r="F14" s="30">
         <v>3</v>
       </c>
       <c r="G14" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>688.5</v>
       </c>
       <c r="I14" s="28"/>
@@ -4926,14 +4959,14 @@
         <v>249.9</v>
       </c>
       <c r="E15" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>224.91</v>
       </c>
       <c r="F15" s="30">
         <v>1</v>
       </c>
       <c r="G15" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>224.91</v>
       </c>
       <c r="I15" s="28"/>
@@ -4952,14 +4985,14 @@
         <v>249.9</v>
       </c>
       <c r="E16" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>224.91</v>
       </c>
       <c r="F16" s="30">
         <v>1</v>
       </c>
       <c r="G16" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>224.91</v>
       </c>
       <c r="I16" s="28"/>
@@ -4978,14 +5011,14 @@
         <v>249.9</v>
       </c>
       <c r="E17" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>224.91</v>
       </c>
       <c r="F17" s="30">
         <v>5</v>
       </c>
       <c r="G17" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>1124.55</v>
       </c>
       <c r="I17" s="28"/>
@@ -5004,14 +5037,14 @@
         <v>199.9</v>
       </c>
       <c r="E18" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>179.91</v>
       </c>
       <c r="F18" s="30">
         <v>0</v>
       </c>
       <c r="G18" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>0</v>
       </c>
       <c r="I18" s="28"/>
@@ -5030,14 +5063,14 @@
         <v>146</v>
       </c>
       <c r="E19" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>131.4</v>
       </c>
       <c r="F19" s="30">
         <v>2</v>
       </c>
       <c r="G19" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>262.8</v>
       </c>
       <c r="I19" s="28"/>
@@ -5056,14 +5089,14 @@
         <v>145</v>
       </c>
       <c r="E20" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>130.5</v>
       </c>
       <c r="F20" s="30">
         <v>2</v>
       </c>
       <c r="G20" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>261</v>
       </c>
       <c r="I20" s="28"/>
@@ -5082,14 +5115,14 @@
         <v>142.9</v>
       </c>
       <c r="E21" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>128.61000000000001</v>
       </c>
       <c r="F21" s="30">
         <v>2</v>
       </c>
       <c r="G21" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>257.22000000000003</v>
       </c>
       <c r="I21" s="28"/>
@@ -5108,14 +5141,14 @@
         <v>140</v>
       </c>
       <c r="E22" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>126</v>
       </c>
       <c r="F22" s="30">
         <v>2</v>
       </c>
       <c r="G22" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>252</v>
       </c>
       <c r="I22" s="28"/>
@@ -5134,14 +5167,14 @@
         <v>93.5</v>
       </c>
       <c r="E23" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>84.15</v>
       </c>
       <c r="F23" s="30">
         <v>2</v>
       </c>
       <c r="G23" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>168.3</v>
       </c>
       <c r="I23" s="28"/>
@@ -5160,14 +5193,14 @@
         <v>92.9</v>
       </c>
       <c r="E24" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>83.61</v>
       </c>
       <c r="F24" s="30">
         <v>6</v>
       </c>
       <c r="G24" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>501.65999999999997</v>
       </c>
     </row>
@@ -5185,14 +5218,14 @@
         <v>91.4</v>
       </c>
       <c r="E25" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>82.26</v>
       </c>
       <c r="F25" s="30">
         <v>2</v>
       </c>
       <c r="G25" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>164.52</v>
       </c>
     </row>
@@ -5210,14 +5243,14 @@
         <v>89.9</v>
       </c>
       <c r="E26" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>80.910000000000011</v>
       </c>
       <c r="F26" s="30">
         <v>5</v>
       </c>
       <c r="G26" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>404.55000000000007</v>
       </c>
     </row>
@@ -5235,14 +5268,14 @@
         <v>89.9</v>
       </c>
       <c r="E27" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>80.910000000000011</v>
       </c>
       <c r="F27" s="30">
         <v>3</v>
       </c>
       <c r="G27" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>242.73000000000002</v>
       </c>
     </row>
@@ -5260,14 +5293,14 @@
         <v>85.9</v>
       </c>
       <c r="E28" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>77.31</v>
       </c>
       <c r="F28" s="30">
         <v>8</v>
       </c>
       <c r="G28" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>618.48</v>
       </c>
     </row>
@@ -5285,14 +5318,14 @@
         <v>70.900000000000006</v>
       </c>
       <c r="E29" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>63.81</v>
       </c>
       <c r="F29" s="30">
         <v>0</v>
       </c>
       <c r="G29" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>0</v>
       </c>
     </row>
@@ -5310,14 +5343,14 @@
         <v>69.900000000000006</v>
       </c>
       <c r="E30" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>62.910000000000004</v>
       </c>
       <c r="F30" s="30">
         <v>15</v>
       </c>
       <c r="G30" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>943.65000000000009</v>
       </c>
     </row>
@@ -5335,14 +5368,14 @@
         <v>65.900000000000006</v>
       </c>
       <c r="E31" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>59.31</v>
       </c>
       <c r="F31" s="30">
         <v>12</v>
       </c>
       <c r="G31" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>711.72</v>
       </c>
     </row>
@@ -5360,14 +5393,14 @@
         <v>49.9</v>
       </c>
       <c r="E32" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>44.91</v>
       </c>
       <c r="F32" s="30">
         <v>21</v>
       </c>
       <c r="G32" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>943.1099999999999</v>
       </c>
     </row>
@@ -5385,14 +5418,14 @@
         <v>48.9</v>
       </c>
       <c r="E33" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>44.01</v>
       </c>
       <c r="F33" s="30">
         <v>2</v>
       </c>
       <c r="G33" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>88.02</v>
       </c>
     </row>
@@ -5410,14 +5443,14 @@
         <v>46.9</v>
       </c>
       <c r="E34" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>42.21</v>
       </c>
       <c r="F34" s="30">
         <v>3</v>
       </c>
       <c r="G34" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>126.63</v>
       </c>
     </row>
@@ -5435,14 +5468,14 @@
         <v>44.9</v>
       </c>
       <c r="E35" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>40.409999999999997</v>
       </c>
       <c r="F35" s="30">
         <v>5</v>
       </c>
       <c r="G35" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>202.04999999999998</v>
       </c>
     </row>
@@ -5460,14 +5493,14 @@
         <v>42.5</v>
       </c>
       <c r="E36" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>38.25</v>
       </c>
       <c r="F36" s="30">
         <v>6</v>
       </c>
       <c r="G36" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>229.5</v>
       </c>
     </row>
@@ -5485,14 +5518,14 @@
         <v>39.9</v>
       </c>
       <c r="E37" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>35.909999999999997</v>
       </c>
       <c r="F37" s="30">
         <v>12</v>
       </c>
       <c r="G37" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>430.91999999999996</v>
       </c>
     </row>
@@ -5510,14 +5543,14 @@
         <v>39.9</v>
       </c>
       <c r="E38" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>35.909999999999997</v>
       </c>
       <c r="F38" s="30">
         <v>10</v>
       </c>
       <c r="G38" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>359.09999999999997</v>
       </c>
     </row>
@@ -5535,14 +5568,14 @@
         <v>39.9</v>
       </c>
       <c r="E39" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>35.909999999999997</v>
       </c>
       <c r="F39" s="30">
         <v>11</v>
       </c>
       <c r="G39" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>395.01</v>
       </c>
     </row>
@@ -5560,14 +5593,14 @@
         <v>32.9</v>
       </c>
       <c r="E40" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>29.61</v>
       </c>
       <c r="F40" s="30">
         <v>6</v>
       </c>
       <c r="G40" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>177.66</v>
       </c>
     </row>
@@ -5585,14 +5618,14 @@
         <v>29.9</v>
       </c>
       <c r="E41" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>26.909999999999997</v>
       </c>
       <c r="F41" s="30">
         <v>10</v>
       </c>
       <c r="G41" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>269.09999999999997</v>
       </c>
     </row>
@@ -5610,14 +5643,14 @@
         <v>25.9</v>
       </c>
       <c r="E42" s="31">
-        <f>Tabela1[[#This Row],[Preço Unitário]]-(Tabela1[[#This Row],[Preço Unitário]]*$I$4)</f>
+        <f>TB_Produtos[[#This Row],[Preço Unitário]]-(TB_Produtos[[#This Row],[Preço Unitário]]*$I$4)</f>
         <v>23.31</v>
       </c>
       <c r="F42" s="30">
         <v>12</v>
       </c>
       <c r="G42" s="31">
-        <f>Tabela1[[#This Row],[Qtd]]*Tabela1[[#This Row],[Preço c/ Desconto]]</f>
+        <f>TB_Produtos[[#This Row],[Qtd]]*TB_Produtos[[#This Row],[Preço c/ Desconto]]</f>
         <v>279.71999999999997</v>
       </c>
     </row>
@@ -5627,23 +5660,23 @@
       </c>
       <c r="B43" s="30"/>
       <c r="C43" s="30">
-        <f>SUBTOTAL(103,Tabela1[Categoria])</f>
+        <f>SUBTOTAL(103,TB_Produtos[Categoria])</f>
         <v>39</v>
       </c>
       <c r="D43" s="33">
-        <f>SUBTOTAL(109,Tabela1[Preço Unitário])</f>
+        <f>SUBTOTAL(109,TB_Produtos[Preço Unitário])</f>
         <v>5962.2999999999938</v>
       </c>
       <c r="E43" s="33">
-        <f>SUBTOTAL(109,Tabela1[Preço c/ Desconto])</f>
+        <f>SUBTOTAL(109,TB_Produtos[Preço c/ Desconto])</f>
         <v>5366.0699999999979</v>
       </c>
       <c r="F43" s="30">
-        <f>SUBTOTAL(109,Tabela1[Qtd])</f>
+        <f>SUBTOTAL(109,TB_Produtos[Qtd])</f>
         <v>183</v>
       </c>
       <c r="G43" s="33">
-        <f>SUBTOTAL(109,Tabela1[Valor Total])</f>
+        <f>SUBTOTAL(109,TB_Produtos[Valor Total])</f>
         <v>14552.549999999997</v>
       </c>
     </row>
@@ -5660,6 +5693,102 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A26CB77B-F399-4629-A253-A85287BD86FF}">
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="4" width="22" customWidth="1"/>
+    <col min="6" max="7" width="22" customWidth="1"/>
+    <col min="8" max="8" width="24.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="35" customFormat="1" ht="29.25" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+    </row>
+    <row r="2" spans="1:9" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="49" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
+      <c r="F2" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="42"/>
+      <c r="H2" s="43"/>
+    </row>
+    <row r="3" spans="1:9" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="F3" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="63.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="36">
+        <f>COUNTA(TB_Produtos[Produtos])</f>
+        <v>39</v>
+      </c>
+      <c r="C4" s="36">
+        <f>SUM(TB_Produtos[Qtd])</f>
+        <v>183</v>
+      </c>
+      <c r="D4" s="52">
+        <f>AVERAGE(TB_Produtos[Qtd])</f>
+        <v>4.6923076923076925</v>
+      </c>
+      <c r="F4" s="36">
+        <f>COUNTIF(TB_Produtos[Produtos],F2)</f>
+        <v>3</v>
+      </c>
+      <c r="G4" s="36">
+        <f>SUMIF(TB_Produtos[Produtos],F2,TB_Produtos[Qtd])</f>
+        <v>4</v>
+      </c>
+      <c r="H4" s="52">
+        <f>AVERAGEIF(TB_Produtos[Produtos],F2,TB_Produtos[Qtd])</f>
+        <v>1.3333333333333333</v>
+      </c>
+      <c r="I4" s="54"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
+  </mergeCells>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Erro de Digitação" error="Este produto não está listado na tabela original." promptTitle="Mensagem de Entrada" prompt="Teste de mensagem de entrada._x000a_" sqref="F2" xr:uid="{8FE46A23-BE40-450F-BCB7-5F3E85C1378C}">
+      <formula1>Int_Nome_Produtos</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BBE6E77-EBCD-448B-AB61-14EA4DC9C25B}">
   <dimension ref="B2:H14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>